<commit_message>
Keep one pie on the A/R pivot sheet: scheduled vs not.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/AR-Sample-Ledger.xlsx
+++ b/AR-Sample-Ledger.xlsx
@@ -11,7 +11,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calcs" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aging pivot" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ledger'!$A$1:$R$111</definedName>
@@ -28,7 +27,7 @@
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,15 +63,6 @@
       <b val="1"/>
       <color rgb="001B365D"/>
       <sz val="13"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001B365D"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <color rgb="001B365D"/>
-      <sz val="14"/>
     </font>
   </fonts>
   <fills count="3">
@@ -114,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -137,9 +127,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -238,129 +225,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Open A/R by aging bucket</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="stacked"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Calcs'!B16</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Calcs'!$A$17:$A$20</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Calcs'!$B$17:$B$20</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Calcs'!C16</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Calcs'!$A$17:$A$20</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Calcs'!$C$17:$C$20</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Dollars</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Patient vs insurance</a:t>
+              <a:t>Patients scheduled vs not scheduled</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -372,6 +237,11 @@
         <ser>
           <idx val="0"/>
           <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Aging pivot'!B31</f>
+            </strRef>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -379,17 +249,18 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Calcs'!$A$6:$A$7</f>
+              <f>'Aging pivot'!$A$32:$A$33</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Calcs'!$B$6:$B$7</f>
+              <f>'Aging pivot'!$B$32:$B$33</f>
             </numRef>
           </val>
         </ser>
         <dLbls>
-          <showVal val="0"/>
+          <showVal val="1"/>
+          <showCatName val="1"/>
           <showPercent val="1"/>
         </dLbls>
         <firstSliceAng val="0"/>
@@ -404,99 +275,16 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="12"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Accounts by primary bucket</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Aging pivot'!D4</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Aging pivot'!$A$5:$A$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Aging pivot'!$D$5:$D$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>0</col>
+      <col>5</col>
       <colOff>0</colOff>
-      <row>7</row>
+      <row>29</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2880000"/>
+    <ext cx="5040000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -506,50 +294,6 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>8</col>
-      <colOff>0</colOff>
-      <row>7</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="4320000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>23</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5400000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="3" name="Chart 3"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -929,7 +673,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ledger · Calcs · Aging pivot · Dashboard</t>
+          <t>Ledger · Calcs · Aging pivot (tables + pie)</t>
         </is>
       </c>
     </row>
@@ -8420,11 +8164,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -8636,10 +8380,6 @@
         <f>SUMIF(Ledger!A:A,A14,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D14" s="13">
-        <f>SUMIF(Ledger!A:A,A14,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8655,10 +8395,6 @@
         <f>SUMIF(Ledger!A:A,A15,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D15" s="13">
-        <f>SUMIF(Ledger!A:A,A15,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8674,10 +8410,6 @@
         <f>SUMIF(Ledger!A:A,A16,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D16" s="13">
-        <f>SUMIF(Ledger!A:A,A16,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -8693,10 +8425,6 @@
         <f>SUMIF(Ledger!A:A,A17,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D17" s="13">
-        <f>SUMIF(Ledger!A:A,A17,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8712,10 +8440,6 @@
         <f>SUMIF(Ledger!A:A,A18,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D18" s="13">
-        <f>SUMIF(Ledger!A:A,A18,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -8731,10 +8455,6 @@
         <f>SUMIF(Ledger!A:A,A19,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D19" s="13">
-        <f>SUMIF(Ledger!A:A,A19,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8750,10 +8470,6 @@
         <f>SUMIF(Ledger!A:A,A20,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D20" s="13">
-        <f>SUMIF(Ledger!A:A,A20,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8769,10 +8485,6 @@
         <f>SUMIF(Ledger!A:A,A21,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D21" s="13">
-        <f>SUMIF(Ledger!A:A,A21,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8788,10 +8500,6 @@
         <f>SUMIF(Ledger!A:A,A22,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D22" s="13">
-        <f>SUMIF(Ledger!A:A,A22,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8807,10 +8515,6 @@
         <f>SUMIF(Ledger!A:A,A23,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D23" s="13">
-        <f>SUMIF(Ledger!A:A,A23,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8826,10 +8530,6 @@
         <f>SUMIF(Ledger!A:A,A24,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D24" s="13">
-        <f>SUMIF(Ledger!A:A,A24,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8845,10 +8545,6 @@
         <f>SUMIF(Ledger!A:A,A25,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D25" s="13">
-        <f>SUMIF(Ledger!A:A,A25,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8864,10 +8560,6 @@
         <f>SUMIF(Ledger!A:A,A26,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D26" s="13">
-        <f>SUMIF(Ledger!A:A,A26,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8883,10 +8575,6 @@
         <f>SUMIF(Ledger!A:A,A27,Ledger!F:F)</f>
         <v/>
       </c>
-      <c r="D27" s="13">
-        <f>SUMIF(Ledger!A:A,A27,Ledger!G:G)</f>
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8904,6 +8592,92 @@
       </c>
       <c r="D28" s="13">
         <f>SUMIF(Ledger!A:A,A28,Ledger!G:G)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Next appointment</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Open $</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="B32">
+        <f>COUNTIF(Ledger!Q2:Q111,"Yes")</f>
+        <v/>
+      </c>
+      <c r="C32" s="13">
+        <f>SUMIF(Ledger!Q2:Q111,"Yes",Ledger!E2:E111)</f>
+        <v/>
+      </c>
+      <c r="D32" s="14">
+        <f>IF($B$34=0,0,B32/$B$34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Not scheduled</t>
+        </is>
+      </c>
+      <c r="B33">
+        <f>COUNTIF(Ledger!Q2:Q111,"No")</f>
+        <v/>
+      </c>
+      <c r="C33" s="13">
+        <f>SUMIF(Ledger!Q2:Q111,"No",Ledger!E2:E111)</f>
+        <v/>
+      </c>
+      <c r="D33" s="14">
+        <f>IF($B$34=0,0,B33/$B$34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B34" s="12">
+        <f>SUM(B32:B33)</f>
+        <v/>
+      </c>
+      <c r="C34" s="16">
+        <f>SUM(C32:C33)</f>
+        <v/>
+      </c>
+      <c r="D34" s="17">
+        <f>SUM(D32:D33)</f>
         <v/>
       </c>
     </row>
@@ -8912,78 +8686,6 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00294BEF"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>Huddle dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Total owing</t>
-        </is>
-      </c>
-      <c r="B3" s="19">
-        <f>Calcs!B5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Patient / insurance</t>
-        </is>
-      </c>
-      <c r="B4" s="20">
-        <f>TEXT(Calcs!B6,"$#,##0")&amp;" / "&amp;TEXT(Calcs!B7,"$#,##0")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Patient 90+</t>
-        </is>
-      </c>
-      <c r="B5" s="19">
-        <f>Calcs!B9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>90+ with no next appointment</t>
-        </is>
-      </c>
-      <c r="B6" s="20">
-        <f>Calcs!B12&amp;" accounts · "&amp;TEXT(Calcs!B25,"$#,##0")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update the public A/R sample with the latest tracker workbook.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/AR-Sample-Ledger.xlsx
+++ b/AR-Sample-Ledger.xlsx
@@ -8,22 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/haley/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DA5E80C-7428-CA45-8E00-40CE58A04F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CDD0F7AA-98D4-6C4A-B65B-049D445866B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Ledger" sheetId="2" r:id="rId1"/>
+    <sheet name="DATA" sheetId="2" r:id="rId1"/>
     <sheet name="About" sheetId="1" r:id="rId2"/>
     <sheet name="Calculations" sheetId="3" r:id="rId3"/>
     <sheet name="Aging pivot" sheetId="4" r:id="rId4"/>
     <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Ledger!$A$1:$R$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DATA!$A$1:$R$111</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -822,6 +821,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF1A355D"/>
+      <color rgb="FF99E3EB"/>
       <color rgb="FF1AD0FF"/>
       <color rgb="FF00FF7A"/>
       <color rgb="FFFFA975"/>
@@ -1957,7 +1958,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
-    <tabColor rgb="FF1B365D"/>
+    <tabColor rgb="FF1A355D"/>
   </sheetPr>
   <dimension ref="A1:R111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2101,7 +2102,7 @@
       </c>
       <c r="D3" s="6">
         <f ca="1">TODAY()+54</f>
-        <v>46366</v>
+        <v>46369</v>
       </c>
       <c r="E3" s="7">
         <v>53.4</v>
@@ -2379,7 +2380,7 @@
       </c>
       <c r="D8" s="6">
         <f ca="1">TODAY()+29</f>
-        <v>46341</v>
+        <v>46344</v>
       </c>
       <c r="E8" s="7">
         <v>95</v>
@@ -2932,7 +2933,7 @@
       </c>
       <c r="D18" s="6">
         <f ca="1">TODAY()+29</f>
-        <v>46341</v>
+        <v>46344</v>
       </c>
       <c r="E18" s="7">
         <v>40.049999999999997</v>
@@ -3045,7 +3046,7 @@
       </c>
       <c r="D20" s="6">
         <f ca="1">TODAY()+23</f>
-        <v>46335</v>
+        <v>46338</v>
       </c>
       <c r="E20" s="7">
         <v>30</v>
@@ -3103,7 +3104,7 @@
       </c>
       <c r="D21" s="6">
         <f ca="1">TODAY()+29</f>
-        <v>46341</v>
+        <v>46344</v>
       </c>
       <c r="E21" s="7">
         <v>195</v>
@@ -3161,7 +3162,7 @@
       </c>
       <c r="D22" s="6">
         <f ca="1">TODAY()+20</f>
-        <v>46332</v>
+        <v>46335</v>
       </c>
       <c r="E22" s="7">
         <v>37</v>
@@ -3219,7 +3220,7 @@
       </c>
       <c r="D23" s="6">
         <f ca="1">TODAY()+59</f>
-        <v>46371</v>
+        <v>46374</v>
       </c>
       <c r="E23" s="7">
         <v>4</v>
@@ -3497,7 +3498,7 @@
       </c>
       <c r="D28" s="6">
         <f ca="1">TODAY()+41</f>
-        <v>46353</v>
+        <v>46356</v>
       </c>
       <c r="E28" s="7">
         <v>14</v>
@@ -3555,7 +3556,7 @@
       </c>
       <c r="D29" s="6">
         <f ca="1">TODAY()+10</f>
-        <v>46322</v>
+        <v>46325</v>
       </c>
       <c r="E29" s="7">
         <v>1431.34</v>
@@ -3723,7 +3724,7 @@
       </c>
       <c r="D32" s="6">
         <f ca="1">TODAY()+24</f>
-        <v>46336</v>
+        <v>46339</v>
       </c>
       <c r="E32" s="7">
         <v>2</v>
@@ -3946,7 +3947,7 @@
       </c>
       <c r="D36" s="6">
         <f ca="1">TODAY()+29</f>
-        <v>46341</v>
+        <v>46344</v>
       </c>
       <c r="E36" s="7">
         <v>233</v>
@@ -4114,7 +4115,7 @@
       </c>
       <c r="D39" s="6">
         <f ca="1">TODAY()+8</f>
-        <v>46320</v>
+        <v>46323</v>
       </c>
       <c r="E39" s="7">
         <v>16</v>
@@ -4337,7 +4338,7 @@
       </c>
       <c r="D43" s="6">
         <f ca="1">TODAY()+54</f>
-        <v>46366</v>
+        <v>46369</v>
       </c>
       <c r="E43" s="7">
         <v>30</v>
@@ -4505,7 +4506,7 @@
       </c>
       <c r="D46" s="6">
         <f ca="1">TODAY()+41</f>
-        <v>46353</v>
+        <v>46356</v>
       </c>
       <c r="E46" s="7">
         <v>30</v>
@@ -4563,7 +4564,7 @@
       </c>
       <c r="D47" s="6">
         <f ca="1">TODAY()+10</f>
-        <v>46322</v>
+        <v>46325</v>
       </c>
       <c r="E47" s="7">
         <v>108.6</v>
@@ -4786,7 +4787,7 @@
       </c>
       <c r="D51" s="6">
         <f ca="1">TODAY()+65</f>
-        <v>46377</v>
+        <v>46380</v>
       </c>
       <c r="E51" s="7">
         <v>50</v>
@@ -5119,7 +5120,7 @@
       </c>
       <c r="D57" s="6">
         <f ca="1">TODAY()+23</f>
-        <v>46335</v>
+        <v>46338</v>
       </c>
       <c r="E57" s="7">
         <v>30.6</v>
@@ -5342,7 +5343,7 @@
       </c>
       <c r="D61" s="6">
         <f ca="1">TODAY()+62</f>
-        <v>46374</v>
+        <v>46377</v>
       </c>
       <c r="E61" s="7">
         <v>107</v>
@@ -5400,7 +5401,7 @@
       </c>
       <c r="D62" s="6">
         <f ca="1">TODAY()+18</f>
-        <v>46330</v>
+        <v>46333</v>
       </c>
       <c r="E62" s="7">
         <v>357</v>
@@ -5568,7 +5569,7 @@
       </c>
       <c r="D65" s="6">
         <f ca="1">TODAY()+36</f>
-        <v>46348</v>
+        <v>46351</v>
       </c>
       <c r="E65" s="7">
         <v>116</v>
@@ -5791,7 +5792,7 @@
       </c>
       <c r="D69" s="6">
         <f ca="1">TODAY()+70</f>
-        <v>46382</v>
+        <v>46385</v>
       </c>
       <c r="E69" s="7">
         <v>50</v>
@@ -5849,7 +5850,7 @@
       </c>
       <c r="D70" s="6">
         <f ca="1">TODAY()+31</f>
-        <v>46343</v>
+        <v>46346</v>
       </c>
       <c r="E70" s="7">
         <v>20.8</v>
@@ -5962,7 +5963,7 @@
       </c>
       <c r="D72" s="6">
         <f ca="1">TODAY()+10</f>
-        <v>46322</v>
+        <v>46325</v>
       </c>
       <c r="E72" s="7">
         <v>311</v>
@@ -6130,7 +6131,7 @@
       </c>
       <c r="D75" s="6">
         <f ca="1">TODAY()+23</f>
-        <v>46335</v>
+        <v>46338</v>
       </c>
       <c r="E75" s="7">
         <v>208</v>
@@ -6188,7 +6189,7 @@
       </c>
       <c r="D76" s="6">
         <f ca="1">TODAY()+17</f>
-        <v>46329</v>
+        <v>46332</v>
       </c>
       <c r="E76" s="7">
         <v>30</v>
@@ -6246,7 +6247,7 @@
       </c>
       <c r="D77" s="6">
         <f ca="1">TODAY()+42</f>
-        <v>46354</v>
+        <v>46357</v>
       </c>
       <c r="E77" s="7">
         <v>3180</v>
@@ -6689,7 +6690,7 @@
       </c>
       <c r="D85" s="6">
         <f ca="1">TODAY()+37</f>
-        <v>46349</v>
+        <v>46352</v>
       </c>
       <c r="E85" s="7">
         <v>208</v>
@@ -6802,7 +6803,7 @@
       </c>
       <c r="D87" s="6">
         <f ca="1">TODAY()+10</f>
-        <v>46322</v>
+        <v>46325</v>
       </c>
       <c r="E87" s="7">
         <v>10.5</v>
@@ -7025,7 +7026,7 @@
       </c>
       <c r="D91" s="6">
         <f ca="1">TODAY()+28</f>
-        <v>46340</v>
+        <v>46343</v>
       </c>
       <c r="E91" s="7">
         <v>21.2</v>
@@ -7138,7 +7139,7 @@
       </c>
       <c r="D93" s="6">
         <f ca="1">TODAY()+41</f>
-        <v>46353</v>
+        <v>46356</v>
       </c>
       <c r="E93" s="7">
         <v>117</v>
@@ -7196,7 +7197,7 @@
       </c>
       <c r="D94" s="6">
         <f ca="1">TODAY()+14</f>
-        <v>46326</v>
+        <v>46329</v>
       </c>
       <c r="E94" s="7">
         <v>28.6</v>
@@ -7584,7 +7585,7 @@
       </c>
       <c r="D101" s="6">
         <f ca="1">TODAY()+64</f>
-        <v>46376</v>
+        <v>46379</v>
       </c>
       <c r="E101" s="7">
         <v>59.6</v>
@@ -7642,7 +7643,7 @@
       </c>
       <c r="D102" s="6">
         <f ca="1">TODAY()+59</f>
-        <v>46371</v>
+        <v>46374</v>
       </c>
       <c r="E102" s="7">
         <v>1549</v>
@@ -7810,7 +7811,7 @@
       </c>
       <c r="D105" s="6">
         <f ca="1">TODAY()+66</f>
-        <v>46378</v>
+        <v>46381</v>
       </c>
       <c r="E105" s="7">
         <v>49.8</v>
@@ -7868,7 +7869,7 @@
       </c>
       <c r="D106" s="6">
         <f ca="1">TODAY()+47</f>
-        <v>46359</v>
+        <v>46362</v>
       </c>
       <c r="E106" s="7">
         <v>21.8</v>
@@ -7981,7 +7982,7 @@
       </c>
       <c r="D108" s="6">
         <f ca="1">TODAY()+63</f>
-        <v>46375</v>
+        <v>46378</v>
       </c>
       <c r="E108" s="7">
         <v>30</v>
@@ -8039,7 +8040,7 @@
       </c>
       <c r="D109" s="6">
         <f ca="1">TODAY()+15</f>
-        <v>46327</v>
+        <v>46330</v>
       </c>
       <c r="E109" s="7">
         <v>51</v>
@@ -8097,7 +8098,7 @@
       </c>
       <c r="D110" s="6">
         <f ca="1">TODAY()+11</f>
-        <v>46323</v>
+        <v>46326</v>
       </c>
       <c r="E110" s="7">
         <v>69</v>
@@ -8155,7 +8156,7 @@
       </c>
       <c r="D111" s="6">
         <f ca="1">TODAY()+13</f>
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="E111" s="7">
         <v>27.5</v>
@@ -8214,6 +8215,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <tabColor theme="0"/>
+  </sheetPr>
   <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -8326,7 +8330,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
-    <tabColor rgb="FF294BEF"/>
+    <tabColor rgb="FF1A355D"/>
   </sheetPr>
   <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -8356,7 +8360,7 @@
         <v>172</v>
       </c>
       <c r="B4">
-        <f>COUNTA(Ledger!B2:B111)</f>
+        <f>COUNTA(DATA!B2:B111)</f>
         <v>110</v>
       </c>
     </row>
@@ -8365,7 +8369,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="12">
-        <f>SUM(Ledger!E2:E111)</f>
+        <f>SUM(DATA!E2:E111)</f>
         <v>22550.509999999991</v>
       </c>
     </row>
@@ -8374,7 +8378,7 @@
         <v>173</v>
       </c>
       <c r="B6" s="12">
-        <f>SUM(Ledger!F2:F111)</f>
+        <f>SUM(DATA!F2:F111)</f>
         <v>20022.139999999996</v>
       </c>
     </row>
@@ -8383,7 +8387,7 @@
         <v>174</v>
       </c>
       <c r="B7" s="12">
-        <f>SUM(Ledger!G2:G111)</f>
+        <f>SUM(DATA!G2:G111)</f>
         <v>2528.37</v>
       </c>
     </row>
@@ -8401,7 +8405,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="12">
-        <f>SUM(Ledger!K2:K111)</f>
+        <f>SUM(DATA!K2:K111)</f>
         <v>20022.139999999996</v>
       </c>
     </row>
@@ -8419,7 +8423,7 @@
         <v>177</v>
       </c>
       <c r="B11">
-        <f>COUNTIF(Ledger!K2:K111,"&gt;0")</f>
+        <f>COUNTIF(DATA!K2:K111,"&gt;0")</f>
         <v>109</v>
       </c>
     </row>
@@ -8428,7 +8432,7 @@
         <v>178</v>
       </c>
       <c r="B12">
-        <f>COUNTIFS(Ledger!K2:K111,"&gt;0",Ledger!Q2:Q111,"No")</f>
+        <f>COUNTIFS(DATA!K2:K111,"&gt;0",DATA!Q2:Q111,"No")</f>
         <v>71</v>
       </c>
     </row>
@@ -8437,7 +8441,7 @@
         <v>179</v>
       </c>
       <c r="B13" s="14">
-        <f>SUMPRODUCT(1/COUNTIF(Ledger!A2:A111,Ledger!A2:A111))</f>
+        <f>SUMPRODUCT(1/COUNTIF(DATA!A2:A111,DATA!A2:A111))</f>
         <v>59.000000000000028</v>
       </c>
     </row>
@@ -8468,11 +8472,11 @@
         <v>186</v>
       </c>
       <c r="B17" s="12">
-        <f>SUM(Ledger!H2:H111)</f>
+        <f>SUM(DATA!H2:H111)</f>
         <v>0</v>
       </c>
       <c r="C17" s="12">
-        <f>SUM(Ledger!L2:L111)</f>
+        <f>SUM(DATA!L2:L111)</f>
         <v>0</v>
       </c>
       <c r="D17" s="12">
@@ -8489,11 +8493,11 @@
         <v>187</v>
       </c>
       <c r="B18" s="12">
-        <f>SUM(Ledger!I2:I111)</f>
+        <f>SUM(DATA!I2:I111)</f>
         <v>0</v>
       </c>
       <c r="C18" s="12">
-        <f>SUM(Ledger!M2:M111)</f>
+        <f>SUM(DATA!M2:M111)</f>
         <v>0</v>
       </c>
       <c r="D18" s="12">
@@ -8510,11 +8514,11 @@
         <v>188</v>
       </c>
       <c r="B19" s="12">
-        <f>SUM(Ledger!J2:J111)</f>
+        <f>SUM(DATA!J2:J111)</f>
         <v>0</v>
       </c>
       <c r="C19" s="12">
-        <f>SUM(Ledger!N2:N111)</f>
+        <f>SUM(DATA!N2:N111)</f>
         <v>0</v>
       </c>
       <c r="D19" s="12">
@@ -8531,11 +8535,11 @@
         <v>21</v>
       </c>
       <c r="B20" s="12">
-        <f>SUM(Ledger!K2:K111)</f>
+        <f>SUM(DATA!K2:K111)</f>
         <v>20022.139999999996</v>
       </c>
       <c r="C20" s="12">
-        <f>SUM(Ledger!O2:O111)</f>
+        <f>SUM(DATA!O2:O111)</f>
         <v>2528.37</v>
       </c>
       <c r="D20" s="12">
@@ -8587,7 +8591,7 @@
         <v>192</v>
       </c>
       <c r="B25" s="12">
-        <f>SUMIFS(Ledger!E2:E111,Ledger!K2:K111,"&gt;0",Ledger!Q2:Q111,"No")</f>
+        <f>SUMIFS(DATA!E2:E111,DATA!K2:K111,"&gt;0",DATA!Q2:Q111,"No")</f>
         <v>13527.720000000003</v>
       </c>
     </row>
@@ -8602,7 +8606,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
-    <tabColor rgb="FFFF88CF"/>
+    <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -8647,19 +8651,19 @@
         <v>186</v>
       </c>
       <c r="B5" s="12">
-        <f>SUMIF(Ledger!P:P,A5,Ledger!F:F)</f>
+        <f>SUMIF(DATA!P:P,A5,DATA!F:F)</f>
         <v>0</v>
       </c>
       <c r="C5" s="12">
-        <f>SUMIF(Ledger!P:P,A5,Ledger!G:G)</f>
+        <f>SUMIF(DATA!P:P,A5,DATA!G:G)</f>
         <v>0</v>
       </c>
       <c r="D5">
-        <f>COUNTIF(Ledger!P:P,A5)</f>
+        <f>COUNTIF(DATA!P:P,A5)</f>
         <v>0</v>
       </c>
       <c r="E5">
-        <f>COUNTIFS(Ledger!P:P,A5,Ledger!Q:Q,"No")</f>
+        <f>COUNTIFS(DATA!P:P,A5,DATA!Q:Q,"No")</f>
         <v>0</v>
       </c>
     </row>
@@ -8668,19 +8672,19 @@
         <v>187</v>
       </c>
       <c r="B6" s="12">
-        <f>SUMIF(Ledger!P:P,A6,Ledger!F:F)</f>
+        <f>SUMIF(DATA!P:P,A6,DATA!F:F)</f>
         <v>0</v>
       </c>
       <c r="C6" s="12">
-        <f>SUMIF(Ledger!P:P,A6,Ledger!G:G)</f>
+        <f>SUMIF(DATA!P:P,A6,DATA!G:G)</f>
         <v>0</v>
       </c>
       <c r="D6">
-        <f>COUNTIF(Ledger!P:P,A6)</f>
+        <f>COUNTIF(DATA!P:P,A6)</f>
         <v>0</v>
       </c>
       <c r="E6">
-        <f>COUNTIFS(Ledger!P:P,A6,Ledger!Q:Q,"No")</f>
+        <f>COUNTIFS(DATA!P:P,A6,DATA!Q:Q,"No")</f>
         <v>0</v>
       </c>
     </row>
@@ -8689,19 +8693,19 @@
         <v>188</v>
       </c>
       <c r="B7" s="12">
-        <f>SUMIF(Ledger!P:P,A7,Ledger!F:F)</f>
+        <f>SUMIF(DATA!P:P,A7,DATA!F:F)</f>
         <v>0</v>
       </c>
       <c r="C7" s="12">
-        <f>SUMIF(Ledger!P:P,A7,Ledger!G:G)</f>
+        <f>SUMIF(DATA!P:P,A7,DATA!G:G)</f>
         <v>0</v>
       </c>
       <c r="D7">
-        <f>COUNTIF(Ledger!P:P,A7)</f>
+        <f>COUNTIF(DATA!P:P,A7)</f>
         <v>0</v>
       </c>
       <c r="E7">
-        <f>COUNTIFS(Ledger!P:P,A7,Ledger!Q:Q,"No")</f>
+        <f>COUNTIFS(DATA!P:P,A7,DATA!Q:Q,"No")</f>
         <v>0</v>
       </c>
     </row>
@@ -8710,19 +8714,19 @@
         <v>21</v>
       </c>
       <c r="B8" s="12">
-        <f>SUMIF(Ledger!P:P,A8,Ledger!F:F)</f>
+        <f>SUMIF(DATA!P:P,A8,DATA!F:F)</f>
         <v>20022.139999999996</v>
       </c>
       <c r="C8" s="12">
-        <f>SUMIF(Ledger!P:P,A8,Ledger!G:G)</f>
+        <f>SUMIF(DATA!P:P,A8,DATA!G:G)</f>
         <v>2528.37</v>
       </c>
       <c r="D8">
-        <f>COUNTIF(Ledger!P:P,A8)</f>
+        <f>COUNTIF(DATA!P:P,A8)</f>
         <v>110</v>
       </c>
       <c r="E8">
-        <f>COUNTIFS(Ledger!P:P,A8,Ledger!Q:Q,"No")</f>
+        <f>COUNTIFS(DATA!P:P,A8,DATA!Q:Q,"No")</f>
         <v>71</v>
       </c>
     </row>
@@ -8776,15 +8780,15 @@
         <v>98</v>
       </c>
       <c r="B14" s="12">
-        <f>SUMIF(Ledger!A:A,A14,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A14,DATA!E:E)</f>
         <v>4115.32</v>
       </c>
       <c r="C14" s="12">
-        <f>SUMIF(Ledger!A:A,A14,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A14,DATA!F:F)</f>
         <v>3660.32</v>
       </c>
       <c r="D14" s="12">
-        <f>SUMIF(Ledger!A:A,A14,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A14,DATA!G:G)</f>
         <v>455</v>
       </c>
     </row>
@@ -8793,15 +8797,15 @@
         <v>118</v>
       </c>
       <c r="B15" s="12">
-        <f>SUMIF(Ledger!A:A,A15,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A15,DATA!E:E)</f>
         <v>3180</v>
       </c>
       <c r="C15" s="12">
-        <f>SUMIF(Ledger!A:A,A15,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A15,DATA!F:F)</f>
         <v>3180</v>
       </c>
       <c r="D15" s="12">
-        <f>SUMIF(Ledger!A:A,A15,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A15,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -8810,15 +8814,15 @@
         <v>156</v>
       </c>
       <c r="B16" s="12">
-        <f>SUMIF(Ledger!A:A,A16,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A16,DATA!E:E)</f>
         <v>2735.6</v>
       </c>
       <c r="C16" s="12">
-        <f>SUMIF(Ledger!A:A,A16,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A16,DATA!F:F)</f>
         <v>1880.6</v>
       </c>
       <c r="D16" s="12">
-        <f>SUMIF(Ledger!A:A,A16,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A16,DATA!G:G)</f>
         <v>855</v>
       </c>
     </row>
@@ -8827,15 +8831,15 @@
         <v>71</v>
       </c>
       <c r="B17" s="12">
-        <f>SUMIF(Ledger!A:A,A17,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A17,DATA!E:E)</f>
         <v>2226.15</v>
       </c>
       <c r="C17" s="12">
-        <f>SUMIF(Ledger!A:A,A17,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A17,DATA!F:F)</f>
         <v>1228.78</v>
       </c>
       <c r="D17" s="12">
-        <f>SUMIF(Ledger!A:A,A17,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A17,DATA!G:G)</f>
         <v>997.37</v>
       </c>
     </row>
@@ -8844,15 +8848,15 @@
         <v>59</v>
       </c>
       <c r="B18" s="12">
-        <f>SUMIF(Ledger!A:A,A18,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A18,DATA!E:E)</f>
         <v>1880.9399999999998</v>
       </c>
       <c r="C18" s="12">
-        <f>SUMIF(Ledger!A:A,A18,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A18,DATA!F:F)</f>
         <v>1659.9399999999998</v>
       </c>
       <c r="D18" s="12">
-        <f>SUMIF(Ledger!A:A,A18,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A18,DATA!G:G)</f>
         <v>221</v>
       </c>
     </row>
@@ -8861,15 +8865,15 @@
         <v>80</v>
       </c>
       <c r="B19" s="12">
-        <f>SUMIF(Ledger!A:A,A19,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A19,DATA!E:E)</f>
         <v>1350</v>
       </c>
       <c r="C19" s="12">
-        <f>SUMIF(Ledger!A:A,A19,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A19,DATA!F:F)</f>
         <v>1350</v>
       </c>
       <c r="D19" s="12">
-        <f>SUMIF(Ledger!A:A,A19,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A19,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -8878,15 +8882,15 @@
         <v>89</v>
       </c>
       <c r="B20" s="12">
-        <f>SUMIF(Ledger!A:A,A20,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A20,DATA!E:E)</f>
         <v>975.1</v>
       </c>
       <c r="C20" s="12">
-        <f>SUMIF(Ledger!A:A,A20,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A20,DATA!F:F)</f>
         <v>975.1</v>
       </c>
       <c r="D20" s="12">
-        <f>SUMIF(Ledger!A:A,A20,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A20,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -8895,15 +8899,15 @@
         <v>32</v>
       </c>
       <c r="B21" s="12">
-        <f>SUMIF(Ledger!A:A,A21,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A21,DATA!E:E)</f>
         <v>523</v>
       </c>
       <c r="C21" s="12">
-        <f>SUMIF(Ledger!A:A,A21,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A21,DATA!F:F)</f>
         <v>523</v>
       </c>
       <c r="D21" s="12">
-        <f>SUMIF(Ledger!A:A,A21,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A21,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -8912,15 +8916,15 @@
         <v>42</v>
       </c>
       <c r="B22" s="12">
-        <f>SUMIF(Ledger!A:A,A22,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A22,DATA!E:E)</f>
         <v>521.45000000000005</v>
       </c>
       <c r="C22" s="12">
-        <f>SUMIF(Ledger!A:A,A22,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A22,DATA!F:F)</f>
         <v>521.45000000000005</v>
       </c>
       <c r="D22" s="12">
-        <f>SUMIF(Ledger!A:A,A22,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A22,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -8929,15 +8933,15 @@
         <v>64</v>
       </c>
       <c r="B23" s="12">
-        <f>SUMIF(Ledger!A:A,A23,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A23,DATA!E:E)</f>
         <v>459.55</v>
       </c>
       <c r="C23" s="12">
-        <f>SUMIF(Ledger!A:A,A23,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A23,DATA!F:F)</f>
         <v>459.55</v>
       </c>
       <c r="D23" s="12">
-        <f>SUMIF(Ledger!A:A,A23,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A23,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -8946,15 +8950,15 @@
         <v>37</v>
       </c>
       <c r="B24" s="12">
-        <f>SUMIF(Ledger!A:A,A24,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A24,DATA!E:E)</f>
         <v>440.5</v>
       </c>
       <c r="C24" s="12">
-        <f>SUMIF(Ledger!A:A,A24,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A24,DATA!F:F)</f>
         <v>440.5</v>
       </c>
       <c r="D24" s="12">
-        <f>SUMIF(Ledger!A:A,A24,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A24,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -8963,15 +8967,15 @@
         <v>129</v>
       </c>
       <c r="B25" s="12">
-        <f>SUMIF(Ledger!A:A,A25,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A25,DATA!E:E)</f>
         <v>339</v>
       </c>
       <c r="C25" s="12">
-        <f>SUMIF(Ledger!A:A,A25,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A25,DATA!F:F)</f>
         <v>339</v>
       </c>
       <c r="D25" s="12">
-        <f>SUMIF(Ledger!A:A,A25,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A25,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -8980,15 +8984,15 @@
         <v>113</v>
       </c>
       <c r="B26" s="12">
-        <f>SUMIF(Ledger!A:A,A26,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A26,DATA!E:E)</f>
         <v>332.8</v>
       </c>
       <c r="C26" s="12">
-        <f>SUMIF(Ledger!A:A,A26,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A26,DATA!F:F)</f>
         <v>332.8</v>
       </c>
       <c r="D26" s="12">
-        <f>SUMIF(Ledger!A:A,A26,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A26,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -8997,15 +9001,15 @@
         <v>87</v>
       </c>
       <c r="B27" s="12">
-        <f>SUMIF(Ledger!A:A,A27,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A27,DATA!E:E)</f>
         <v>277</v>
       </c>
       <c r="C27" s="12">
-        <f>SUMIF(Ledger!A:A,A27,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A27,DATA!F:F)</f>
         <v>277</v>
       </c>
       <c r="D27" s="12">
-        <f>SUMIF(Ledger!A:A,A27,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A27,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -9014,15 +9018,15 @@
         <v>51</v>
       </c>
       <c r="B28" s="12">
-        <f>SUMIF(Ledger!A:A,A28,Ledger!E:E)</f>
+        <f>SUMIF(DATA!A:A,A28,DATA!E:E)</f>
         <v>272.7</v>
       </c>
       <c r="C28" s="12">
-        <f>SUMIF(Ledger!A:A,A28,Ledger!F:F)</f>
+        <f>SUMIF(DATA!A:A,A28,DATA!F:F)</f>
         <v>272.7</v>
       </c>
       <c r="D28" s="12">
-        <f>SUMIF(Ledger!A:A,A28,Ledger!G:G)</f>
+        <f>SUMIF(DATA!A:A,A28,DATA!G:G)</f>
         <v>0</v>
       </c>
     </row>
@@ -9050,11 +9054,11 @@
         <v>198</v>
       </c>
       <c r="B32">
-        <f>COUNTIF(Ledger!Q2:Q111,"Yes")</f>
+        <f>COUNTIF(DATA!Q2:Q111,"Yes")</f>
         <v>39</v>
       </c>
       <c r="C32" s="12">
-        <f>SUMIF(Ledger!Q2:Q111,"Yes",Ledger!E2:E111)</f>
+        <f>SUMIF(DATA!Q2:Q111,"Yes",DATA!E2:E111)</f>
         <v>9022.7899999999991</v>
       </c>
       <c r="D32" s="13">
@@ -9067,11 +9071,11 @@
         <v>199</v>
       </c>
       <c r="B33">
-        <f>COUNTIF(Ledger!Q2:Q111,"No")</f>
+        <f>COUNTIF(DATA!Q2:Q111,"No")</f>
         <v>71</v>
       </c>
       <c r="C33" s="12">
-        <f>SUMIF(Ledger!Q2:Q111,"No",Ledger!E2:E111)</f>
+        <f>SUMIF(DATA!Q2:Q111,"No",DATA!E2:E111)</f>
         <v>13527.720000000003</v>
       </c>
       <c r="D33" s="13">

</xml_diff>